<commit_message>
Update suffix envelope presentation metrics
</commit_message>
<xml_diff>
--- a/doc/presentation-data/payback_global_suffix_wins_rtx5090_k1m.xlsx
+++ b/doc/presentation-data/payback_global_suffix_wins_rtx5090_k1m.xlsx
@@ -492,14 +492,14 @@
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="39" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Payback-sticky vs. Global Tight Bound vs. Suffix Envelope — RTX 5090, K=1M</t>
+          <t>Momentum vs. Global Tight Bound vs. Suffix Envelope — RTX 5090, K=1M</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Payback-sticky</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -526,12 +526,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Global products avoided</t>
+          <t>Candidate checks avoided (Global / Suffix)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Suffix products avoided</t>
+          <t>PfxtNode materializations avoided (Global / Suffix)</t>
         </is>
       </c>
     </row>
@@ -554,11 +554,15 @@
           <t>70.665 (8.688×)</t>
         </is>
       </c>
-      <c r="E3" s="6" t="n">
-        <v>0.925</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>0.995</v>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>92.5% / 99.5%</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>68.1% / 68.1%</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -580,11 +584,15 @@
           <t>34.727 (1.114×)</t>
         </is>
       </c>
-      <c r="E4" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="10" t="n">
-        <v>0.523</v>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>0.0% / 52.3%</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>0.0% / 0.0%</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -606,11 +614,15 @@
           <t>39.331 (1.095×)</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>0.546</v>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>0.0% / 54.6%</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>0.0% / 0.0%</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -632,11 +644,15 @@
           <t>69.536 (1.081×)</t>
         </is>
       </c>
-      <c r="E6" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="10" t="n">
-        <v>0.334</v>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>1.3% / 34.2%</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>0.0% / 0.0%</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -658,11 +674,15 @@
           <t>56.314 (1.076×)</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n">
-        <v>0.061</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>0.821</v>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>6.1% / 82.1%</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>0.3% / 0.3%</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -684,24 +704,28 @@
           <t>87.376 (1.157×)</t>
         </is>
       </c>
-      <c r="E8" s="10" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="F8" s="10" t="n">
-        <v>0.853</v>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>33.3% / 85.3%</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>10.8% / 10.8%</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Runtime columns are milliseconds; speedups in parentheses are relative to payback-sticky.</t>
+          <t>Runtime columns are milliseconds; speedups in parentheses are relative to Momentum.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Both products-avoided columns are relative to payback-sticky materialized-product counts. Headline timing is cold setup + PFXT.</t>
+          <t>Avoidance is relative to Momentum and shown as Global / Suffix. Headline timing is cold setup + PFXT.</t>
         </is>
       </c>
     </row>

</xml_diff>